<commit_message>
Add support for award coordinates file and enhance error handling in medal showcase
</commit_message>
<xml_diff>
--- a/IL-2_Tracker_award_coordinates.xlsx
+++ b/IL-2_Tracker_award_coordinates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bleih\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40580883-4840-4234-9F86-58168A4659AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F0967A-5FEA-4C38-AF4D-3B17D06D01E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38052" yWindow="4932" windowWidth="21156" windowHeight="18600" xr2:uid="{E6D131E9-51AD-48C7-A8DF-61BD79F7615F}"/>
   </bookViews>
@@ -89,9 +89,6 @@
     <t>red_wound_stripe_big1</t>
   </si>
   <si>
-    <t>Glass_overlay_USSR</t>
-  </si>
-  <si>
     <t>replacements</t>
   </si>
   <si>
@@ -318,6 +315,9 @@
   </si>
   <si>
     <t>Britain_overlay</t>
+  </si>
+  <si>
+    <t>USSR_overlay</t>
   </si>
 </sst>
 </file>
@@ -720,7 +720,7 @@
         <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -914,10 +914,10 @@
         <v>390</v>
       </c>
       <c r="G12" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" t="s">
         <v>19</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -937,12 +937,12 @@
         <v>212</v>
       </c>
       <c r="G13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>93</v>
       </c>
       <c r="B14">
         <v>101</v>
@@ -959,7 +959,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>1</v>
@@ -974,7 +974,7 @@
         <v>9</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
@@ -1164,10 +1164,10 @@
         <v>503</v>
       </c>
       <c r="G27" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" t="s">
         <v>19</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
@@ -1189,7 +1189,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>93</v>
       </c>
       <c r="B29">
         <v>101</v>
@@ -1204,12 +1204,12 @@
         <v>1164</v>
       </c>
       <c r="G29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>1</v>
@@ -1226,7 +1226,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B32">
         <v>156</v>
@@ -1241,24 +1241,24 @@
         <v>455</v>
       </c>
       <c r="G32" t="s">
+        <v>24</v>
+      </c>
+      <c r="H32" t="s">
         <v>25</v>
       </c>
-      <c r="H32" t="s">
+      <c r="I32" t="s">
         <v>26</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>27</v>
       </c>
-      <c r="J32" t="s">
+      <c r="K32" t="s">
         <v>28</v>
-      </c>
-      <c r="K32" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33">
         <v>454</v>
@@ -1273,21 +1273,21 @@
         <v>485</v>
       </c>
       <c r="G33" t="s">
+        <v>30</v>
+      </c>
+      <c r="H33" t="s">
         <v>31</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>32</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>33</v>
-      </c>
-      <c r="J33" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34">
         <v>772</v>
@@ -1302,12 +1302,12 @@
         <v>503</v>
       </c>
       <c r="G34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35">
         <v>1304</v>
@@ -1322,15 +1322,15 @@
         <v>465</v>
       </c>
       <c r="G35" t="s">
+        <v>37</v>
+      </c>
+      <c r="H35" t="s">
         <v>38</v>
-      </c>
-      <c r="H35" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B36">
         <v>1632</v>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B37">
         <v>323</v>
@@ -1362,13 +1362,13 @@
         <v>455</v>
       </c>
       <c r="G37" t="s">
+        <v>41</v>
+      </c>
+      <c r="H37" t="s">
         <v>42</v>
       </c>
-      <c r="H37" t="s">
+      <c r="I37" t="s">
         <v>43</v>
-      </c>
-      <c r="I37" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
@@ -1390,7 +1390,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B39">
         <v>1117</v>
@@ -1405,15 +1405,15 @@
         <v>493</v>
       </c>
       <c r="G39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B40">
         <v>1511</v>
@@ -1428,15 +1428,15 @@
         <v>479</v>
       </c>
       <c r="G40" t="s">
+        <v>48</v>
+      </c>
+      <c r="H40" t="s">
         <v>49</v>
-      </c>
-      <c r="H40" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B41">
         <v>32</v>
@@ -1453,7 +1453,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>1</v>
@@ -1468,12 +1468,12 @@
         <v>9</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B44">
         <v>141</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B45">
         <v>504</v>
@@ -1507,7 +1507,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B46">
         <v>838</v>
@@ -1522,21 +1522,21 @@
         <v>503</v>
       </c>
       <c r="G46" t="s">
+        <v>54</v>
+      </c>
+      <c r="H46" t="s">
         <v>55</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>56</v>
       </c>
-      <c r="I46" t="s">
+      <c r="J46" t="s">
         <v>57</v>
-      </c>
-      <c r="J46" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B47">
         <v>1262</v>
@@ -1553,7 +1553,7 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48">
         <v>1631</v>
@@ -1587,7 +1587,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B50">
         <v>727</v>
@@ -1604,7 +1604,7 @@
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B51">
         <v>1014</v>
@@ -1619,15 +1619,15 @@
         <v>250</v>
       </c>
       <c r="G51" t="s">
+        <v>62</v>
+      </c>
+      <c r="H51" t="s">
         <v>63</v>
-      </c>
-      <c r="H51" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B52">
         <v>1474</v>
@@ -1642,15 +1642,15 @@
         <v>353</v>
       </c>
       <c r="G52" t="s">
+        <v>65</v>
+      </c>
+      <c r="H52" t="s">
         <v>66</v>
-      </c>
-      <c r="H52" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53">
         <v>32</v>
@@ -1667,7 +1667,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>1</v>
@@ -1682,12 +1682,12 @@
         <v>9</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B56">
         <v>178</v>
@@ -1702,15 +1702,15 @@
         <v>494</v>
       </c>
       <c r="G56" t="s">
+        <v>71</v>
+      </c>
+      <c r="H56" t="s">
         <v>72</v>
-      </c>
-      <c r="H56" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B57">
         <v>513</v>
@@ -1725,15 +1725,15 @@
         <v>493</v>
       </c>
       <c r="G57" t="s">
+        <v>74</v>
+      </c>
+      <c r="H57" t="s">
         <v>75</v>
-      </c>
-      <c r="H57" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B58">
         <v>881</v>
@@ -1748,12 +1748,12 @@
         <v>504</v>
       </c>
       <c r="G58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B59">
         <v>1257</v>
@@ -1768,15 +1768,15 @@
         <v>498</v>
       </c>
       <c r="G59" t="s">
+        <v>79</v>
+      </c>
+      <c r="H59" t="s">
         <v>80</v>
-      </c>
-      <c r="H59" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B60">
         <v>1614</v>
@@ -1791,15 +1791,15 @@
         <v>494</v>
       </c>
       <c r="G60" t="s">
+        <v>82</v>
+      </c>
+      <c r="H60" t="s">
         <v>83</v>
-      </c>
-      <c r="H60" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B61">
         <v>124</v>
@@ -1816,7 +1816,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B62">
         <v>580</v>
@@ -1833,7 +1833,7 @@
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B63">
         <v>1073</v>
@@ -1848,15 +1848,15 @@
         <v>284</v>
       </c>
       <c r="G63" t="s">
+        <v>87</v>
+      </c>
+      <c r="H63" t="s">
         <v>88</v>
-      </c>
-      <c r="H63" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B64">
         <v>1597</v>
@@ -1871,15 +1871,15 @@
         <v>497</v>
       </c>
       <c r="G64" t="s">
+        <v>90</v>
+      </c>
+      <c r="H64" t="s">
         <v>91</v>
-      </c>
-      <c r="H64" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B65">
         <v>32</v>

</xml_diff>